<commit_message>
Add Las Vegas Open singles quarterfinals sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013YKMrzX46ZPSCtQnpqcVuf
</commit_message>
<xml_diff>
--- a/las_vegas_quarterfinals.xlsx
+++ b/las_vegas_quarterfinals.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Quarterfinals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Singles QF" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -56,12 +57,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -985,7 +987,557 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Match #</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Player 1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Singles value</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Player 2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Seed</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Singles value</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>P1 game win %</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>P1 match win % (Bo3)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>P2 match win % (Bo3)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Favorite</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mens Singles</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>41</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Luc Pham</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>1.3625</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>John Lucian Goins</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>1.7127</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>0.2016580551917633</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>0.1055966723322519</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>0.8944033276677481</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>John Lucian Goins</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mens Singles</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>42</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Christian Alshon</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>1.9336</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Ben Johns</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>19</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>1.8777</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>0.5531918877057368</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>0.5794868317600381</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>0.4205131682399619</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Christian Alshon</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Mens Singles</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>43</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Federico Staksrud</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>2.0687</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Gabriel Joseph</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>9</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>1.6203</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>0.8583741835725427</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>0.9455078093250174</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>0.05449219067498257</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Federico Staksrud</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Mens Singles</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>44</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hunter Johnson</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>2.0092</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Roscoe Bellamy</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>1.7226</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>0.7542276519342253</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>0.8484791477426963</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>0.1515208522573037</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Hunter Johnson</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Womens Singles</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>31</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Kate Fahey</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>2.0525</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Kiora Kunimoto</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>1.4953</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>0.907369144868414</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>0.9758482075658739</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>0.02415179243412613</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Kate Fahey</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Womens Singles</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>32</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Chao Yi Wang</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>1.3902</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Cailyn Campbell</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>1.1701</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>0.7006234325819415</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>0.7847850581668084</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>0.2152149418331916</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Chao Yi Wang</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Womens Singles</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>33</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Kaitlyn Christian</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>1.6572</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Milan Rane</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>11</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>1.0949</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>0.9089127278599146</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>0.9766208089256847</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>0.0233791910743153</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Kaitlyn Christian</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Womens Singles</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>34</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lea Jansen</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>1.6879</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Genie Bouchard</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>1.459</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>fitted</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>0.7077922568675101</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>0.7937444342523038</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>0.2062555657476962</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Lea Jansen</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -1019,6 +1571,13 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Singles QF sheet: singles suite values (data/singles_players.csv) integrated over both players' sd, race-to-11, best-of-3, NO doubles calibration (same as the live page singles pre-match). Singles values are within-gender; tier = fitted/blended/imputed evidence level.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>